<commit_message>
Added All Activity Diagrams, Fixed Some Mistakes on Use Case Description
</commit_message>
<xml_diff>
--- a/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
+++ b/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\SLC\TPA Desktop\DESKTOP-NB-242\Diagram\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8037362-FEA8-4941-8161-CA87E2D5E8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8210BE4E-4D0A-4F33-92AA-1AF86B0A9A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="4" activeTab="8" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="3" activeTab="7" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
   </bookViews>
   <sheets>
-    <sheet name="TMPLT" sheetId="3" r:id="rId1"/>
-    <sheet name="Edit Restaurant Details" sheetId="1" r:id="rId2"/>
-    <sheet name="Allocate Restaurant Staff" sheetId="5" r:id="rId3"/>
-    <sheet name="Send Broadcast Message" sheetId="8" r:id="rId4"/>
-    <sheet name="Submit Maintenance Report" sheetId="7" r:id="rId5"/>
-    <sheet name="Edit Menu Details" sheetId="2" r:id="rId6"/>
-    <sheet name="Edit Ride Queue" sheetId="4" r:id="rId7"/>
-    <sheet name="Assign Maintenance Tasks" sheetId="10" r:id="rId8"/>
-    <sheet name="Allocate Ride Staff" sheetId="6" r:id="rId9"/>
+    <sheet name="Edit Restaurant Details" sheetId="1" r:id="rId1"/>
+    <sheet name="Allocate Restaurant Staff" sheetId="5" r:id="rId2"/>
+    <sheet name="Send Broadcast Message" sheetId="8" r:id="rId3"/>
+    <sheet name="Submit Maintenance Report" sheetId="7" r:id="rId4"/>
+    <sheet name="Edit Menu Details" sheetId="2" r:id="rId5"/>
+    <sheet name="Edit Ride Queue" sheetId="4" r:id="rId6"/>
+    <sheet name="Assign Maintenance Job" sheetId="10" r:id="rId7"/>
+    <sheet name="Allocate Ride Staff" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="177">
   <si>
     <t>Use Case Name:</t>
   </si>
@@ -139,15 +138,9 @@
     <t>-</t>
   </si>
   <si>
-    <t>4.1. System validates the input.</t>
-  </si>
-  <si>
     <t>1.1. Selected Restaurant doesn't exist.</t>
   </si>
   <si>
-    <t>4.1 User input is invalid.</t>
-  </si>
-  <si>
     <t>Edit Menu Details</t>
   </si>
   <si>
@@ -190,12 +183,6 @@
     <t>1.1. Selected Menu doesn't exist.</t>
   </si>
   <si>
-    <t>4.2. System saves the new restaurant details to database if valid.</t>
-  </si>
-  <si>
-    <t>4.2. System saves the new menu details to database if valid.</t>
-  </si>
-  <si>
     <t>Edit Ride Queue</t>
   </si>
   <si>
@@ -250,9 +237,6 @@
     <t>3.1. System validates changes made to the queue.</t>
   </si>
   <si>
-    <t>3.1 User added to the queue doesn't exist, User added to the queue is already in another/current queue.</t>
-  </si>
-  <si>
     <t>3.2 System updates queue database if changes made are valid.</t>
   </si>
   <si>
@@ -355,45 +339,18 @@
     <t>Maintenance Staff members wants to submit a report to Maintenance Manager.</t>
   </si>
   <si>
-    <t>Maintenance Staff members are able to give a detailed report to their manager regarding the progress/completion of their assigned task.</t>
-  </si>
-  <si>
     <t>Maintenance Staff</t>
   </si>
   <si>
-    <t>1. Maintenance Staff members presses "submit report" while viewing their assigned task.</t>
-  </si>
-  <si>
-    <t>2. Maintenance Staff members want to submit reports upon the completion/progress of their assigned task.</t>
-  </si>
-  <si>
     <t>Maintenance Manager, Ride Manager</t>
   </si>
   <si>
-    <t>View Assigned Maintenance Task must be invoked first before being able to invoke this use case.</t>
-  </si>
-  <si>
     <t>1. User must be logged in as an maintenance staff.</t>
   </si>
   <si>
-    <t>2. User must be assigned a maintenance task.</t>
-  </si>
-  <si>
-    <t>3. User must be viewing said assigned task.</t>
-  </si>
-  <si>
     <t>1. Maintenance Report will be pending review for maintenance manager.</t>
   </si>
   <si>
-    <t>1. User views their assigned task.</t>
-  </si>
-  <si>
-    <t>1.1. System displays their assigned task.</t>
-  </si>
-  <si>
-    <t>1.1 User is currently not assigned a task.</t>
-  </si>
-  <si>
     <t>3. User fills report form according to their progress.</t>
   </si>
   <si>
@@ -412,18 +369,12 @@
     <t>4.2 System saves report into database for manager review.</t>
   </si>
   <si>
-    <t>4.1 Report filled out is invalid.</t>
-  </si>
-  <si>
     <t>Send Broadcast Message</t>
   </si>
   <si>
     <t>Customer Service Manager wants to send a broadcast message.</t>
   </si>
   <si>
-    <t>2. Customer Service Manager wants to send a broadcast message to notify users of an announcement.</t>
-  </si>
-  <si>
     <t>1. Customer Service Manager presses "create broadcast message" button.</t>
   </si>
   <si>
@@ -454,63 +405,18 @@
     <t>4. User presses send broadcast.</t>
   </si>
   <si>
-    <t>4.1 System validates broadcast contents</t>
-  </si>
-  <si>
     <t>4.2 System sends broadcast message to recepients.</t>
   </si>
   <si>
     <t>1.1 System displays broadcast form.</t>
   </si>
   <si>
-    <t>4.1 Broadcast content is invalid.</t>
-  </si>
-  <si>
-    <t>Assign Maintenance Task</t>
-  </si>
-  <si>
-    <t>Maintenance manager wants to assign staff members to a maintenance task.</t>
-  </si>
-  <si>
-    <t>1. User (Maintenance manager) presses the assign staff button while viewing all maintenance tasks.</t>
-  </si>
-  <si>
-    <t>2. User wants to assign maintenance staff to a task to fix the problem.</t>
-  </si>
-  <si>
-    <t>The Maintenance Manager is able to manage Maintenance Division Staff Members such as allocating and de-allocating staff members to tasks depending on importance and damage levels.</t>
-  </si>
-  <si>
     <t>Maintenance Manager</t>
   </si>
   <si>
-    <t>View All Maintenance Tasks must be invoked before invoking this use case.</t>
-  </si>
-  <si>
     <t>1. User must be logged in as an Maintenance manager.</t>
   </si>
   <si>
-    <t>2. There must be at least 1 unassigned/pending maintenance task.</t>
-  </si>
-  <si>
-    <t>1. User views all maintenance tasks page.</t>
-  </si>
-  <si>
-    <t>1.1. System displays all maintenance tasks.</t>
-  </si>
-  <si>
-    <t>1.1 There are no maintenance tasks.</t>
-  </si>
-  <si>
-    <t>2. User selects a maintenance task.</t>
-  </si>
-  <si>
-    <t>2.1 System displays the maintenance task details.</t>
-  </si>
-  <si>
-    <t>3.1. System displays the staff allocated for said task, available staff, and staff assigned in another task.</t>
-  </si>
-  <si>
     <t>5.1 System validates staff assignment list.</t>
   </si>
   <si>
@@ -524,6 +430,150 @@
   </si>
   <si>
     <t>4. User updates staff assignment list according to need and specification.</t>
+  </si>
+  <si>
+    <t>4.5. System saves the new restaurant details to database if valid.</t>
+  </si>
+  <si>
+    <t>4.1. Restaurant Name is empty.</t>
+  </si>
+  <si>
+    <t>4.2. Restaurant Description length is less than 20.</t>
+  </si>
+  <si>
+    <t>4.1. Validate Restaurant Name.</t>
+  </si>
+  <si>
+    <t>4.2. Validate Restaurant Description.</t>
+  </si>
+  <si>
+    <t>4.3. Validate Restaurant Photo.</t>
+  </si>
+  <si>
+    <t>4.4. Validate Operating Hours.</t>
+  </si>
+  <si>
+    <t>4.4. Operating Hours is invalid.</t>
+  </si>
+  <si>
+    <t>4.3. Restaurant Photo not selected.</t>
+  </si>
+  <si>
+    <t>4.1 Unavailable staff assigned, staff already assigned, staff on leave, etc.</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>2. Customer Service Manager wants to send a broadcast message to notify people of an announcement.</t>
+  </si>
+  <si>
+    <t>4.1 Broadcast content is empty.</t>
+  </si>
+  <si>
+    <t>4.1 System validates broadcast content.</t>
+  </si>
+  <si>
+    <t>4.1 Report is empty.</t>
+  </si>
+  <si>
+    <t>1.1 User is currently not assigned to work on a report.</t>
+  </si>
+  <si>
+    <t>3. User must be viewing said assigned report.</t>
+  </si>
+  <si>
+    <t>1. Maintenance Staff members presses "Create report" while viewing their assigned report.</t>
+  </si>
+  <si>
+    <t>2. Maintenance Staff members want to submit reports upon the completion of their assigned job.</t>
+  </si>
+  <si>
+    <t>Maintenance Staff members are able to give a detailed report to their manager regarding the completion of their assigned job.</t>
+  </si>
+  <si>
+    <t>View Assigned Maintenance Job must be invoked first before being able to invoke this use case.</t>
+  </si>
+  <si>
+    <t>2. User must be assigned to work on a report.</t>
+  </si>
+  <si>
+    <t>1. User views their assigned job.</t>
+  </si>
+  <si>
+    <t>1.1. System displays their assigned job.</t>
+  </si>
+  <si>
+    <t>4.1. System validates menu name.</t>
+  </si>
+  <si>
+    <t>4.2. System validates menu description.</t>
+  </si>
+  <si>
+    <t>4.3. System validates menu price.</t>
+  </si>
+  <si>
+    <t>4.4. System validates menu photo.</t>
+  </si>
+  <si>
+    <t>4.1 Menu name is empty.</t>
+  </si>
+  <si>
+    <t>4.2 Menu description length is less than 20</t>
+  </si>
+  <si>
+    <t>4.3 Menu price is less than or equal to 0</t>
+  </si>
+  <si>
+    <t>4.5. System saves the new menu details to database if valid.</t>
+  </si>
+  <si>
+    <t>4.4 Menu Photo is not selected</t>
+  </si>
+  <si>
+    <t>4. User presses save changes.</t>
+  </si>
+  <si>
+    <t>3.1 Customer left queue while staff is editing queue (resulting in customer being re-added to queue if not managed)</t>
+  </si>
+  <si>
+    <t>Assign Maintenance Job</t>
+  </si>
+  <si>
+    <t>Maintenance manager wants to assign staff members to a maintenance Job.</t>
+  </si>
+  <si>
+    <t>1. User (Maintenance manager) presses the assign staff button while viewing all maintenance jobs.</t>
+  </si>
+  <si>
+    <t>2. User wants to assign maintenance staff to a job.</t>
+  </si>
+  <si>
+    <t>The Maintenance Manager is able to manage Maintenance Division Staff Members such as allocating and de-allocating staff members to tasks and reports depending on importance and damage levels.</t>
+  </si>
+  <si>
+    <t>View All Maintenance Jobs must be invoked before invoking this use case.</t>
+  </si>
+  <si>
+    <t>2. There must be at least 1 unassigned/pending maintenance job.</t>
+  </si>
+  <si>
+    <t>1. User views all maintenance job page.</t>
+  </si>
+  <si>
+    <t>2. User selects a maintenance job.</t>
+  </si>
+  <si>
+    <t>1.1. System displays all maintenance jobs.</t>
+  </si>
+  <si>
+    <t>2.1 System displays the maintenance job details.</t>
+  </si>
+  <si>
+    <t>3.1. System displays the staff allocated for said job, available staff, and staff assigned in another job.</t>
+  </si>
+  <si>
+    <t>1.1 There are no maintenance jobs.</t>
   </si>
 </sst>
 </file>
@@ -653,7 +703,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -692,10 +742,34 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -709,30 +783,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -741,6 +791,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1054,172 +1110,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55053E33-AC39-497F-9880-F34198EA3B5F}">
-  <dimension ref="B2:D25"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="17.58203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.4140625" customWidth="1"/>
-    <col min="4" max="4" width="62" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="16"/>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="16"/>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="28"/>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="26"/>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
-    </row>
-    <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="21"/>
-      <c r="D8" s="22"/>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26"/>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="26"/>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="11"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="13"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="16"/>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="C25" s="10"/>
-    </row>
-  </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A3915B7-9862-624A-8796-A82526CFDDED}">
-  <dimension ref="B2:D21"/>
+  <dimension ref="B2:D27"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
@@ -1231,106 +1123,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="16"/>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="16"/>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="16"/>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="28"/>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="16"/>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="16"/>
+      <c r="D8" s="18"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="16"/>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="26"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="16"/>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="26"/>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="16"/>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1341,7 +1233,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1350,7 +1242,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="6" t="s">
         <v>25</v>
       </c>
@@ -1359,7 +1251,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="6" t="s">
         <v>28</v>
       </c>
@@ -1368,39 +1260,95 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>31</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="26"/>
       <c r="C19" s="6"/>
       <c r="D19" s="5" t="s">
-        <v>48</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="26"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="26"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="27"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="16"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="C23" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="18"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="26"/>
+      <c r="C24" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" s="18"/>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B25" s="26"/>
+      <c r="C25" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="18"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B26" s="26"/>
+      <c r="C26" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" s="18"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B27" s="27"/>
+      <c r="C27" s="17" t="s">
+        <v>136</v>
+      </c>
+      <c r="D27" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="21">
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="B14:B22"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B23:B27"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C2:D2"/>
@@ -1408,23 +1356,12 @@
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B9B19F-9F2C-488A-80B2-967228FB8F6A}">
   <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1438,106 +1375,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>74</v>
-      </c>
-      <c r="D5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="16"/>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="16"/>
+      <c r="D8" s="18"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="26"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="16"/>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="26"/>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="16"/>
+      <c r="C13" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -1548,7 +1485,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1557,66 +1494,65 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="16"/>
+      <c r="C20" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="17" t="s">
+        <v>138</v>
+      </c>
+      <c r="D21" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -1624,19 +1560,20 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB3C5E41-754C-46AC-8647-361E83105886}">
-  <dimension ref="B2:D22"/>
+  <dimension ref="B2:D26"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.58203125" bestFit="1" customWidth="1"/>
@@ -1648,92 +1585,92 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="D5" s="16"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="18"/>
     </row>
     <row r="6" spans="2:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="D6" s="22"/>
+      <c r="C6" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="24"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="D7" s="16"/>
+      <c r="C7" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="22"/>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="D10" s="26"/>
+      <c r="C10" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="16"/>
+      <c r="C11" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1744,68 +1681,67 @@
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="18"/>
+      <c r="B13" s="26"/>
       <c r="C13" s="11" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="18"/>
+      <c r="B14" s="26"/>
       <c r="C14" s="12" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="12" t="s">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="12" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="19"/>
+      <c r="B17" s="27"/>
       <c r="C17" s="12"/>
       <c r="D17" s="11" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="D18" s="16"/>
+      <c r="C18" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" s="18"/>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C22" s="10"/>
     </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C26" t="s">
+        <v>139</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B12:B17"/>
     <mergeCell ref="C18:D18"/>
@@ -1813,12 +1749,18 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{433C6673-D655-44ED-B9F0-E1CD3A0F8D79}">
   <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -1832,106 +1774,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="28"/>
-    </row>
-    <row r="6" spans="2:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="22"/>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" s="16"/>
-    </row>
-    <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="18"/>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="D8" s="22"/>
+      <c r="C8" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="26"/>
+      <c r="C10" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="D11" s="16"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="D12" s="26"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="D13" s="16"/>
+      <c r="C13" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -1942,75 +1884,74 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="11" t="s">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="12" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="D20" s="16"/>
+      <c r="C20" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="D21" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2018,19 +1959,20 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259683E5-02D5-4B39-B55A-2E3DAEB07183}">
-  <dimension ref="B2:D25"/>
+  <dimension ref="B2:D29"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.58203125" bestFit="1" customWidth="1"/>
@@ -2042,106 +1984,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="D5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="16"/>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" s="22"/>
+      <c r="C8" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="16"/>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="26"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="16"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="26"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="16"/>
+      <c r="C13" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -2152,25 +2094,25 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="9" t="s">
         <v>25</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="6" t="s">
         <v>28</v>
       </c>
@@ -2179,67 +2121,112 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="29" t="s">
-        <v>29</v>
+        <v>162</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>31</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
-      <c r="C19" s="30"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="34"/>
       <c r="D19" s="5" t="s">
-        <v>49</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="26"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="5" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B21" s="26"/>
+      <c r="C21" s="34"/>
+      <c r="D21" s="5" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B22" s="27"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="5" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B23" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="16"/>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="C23" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="18"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B24" s="26"/>
+      <c r="C24" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="C25" s="10"/>
+      <c r="B25" s="26"/>
+      <c r="C25" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" s="18"/>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B26" s="26"/>
+      <c r="C26" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="D26" s="18"/>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B27" s="27"/>
+      <c r="C27" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="D27" s="18"/>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C29" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="22">
+    <mergeCell ref="B14:B22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B23:B27"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:D10"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C13:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A884BFFD-E428-4208-A11C-6F780788E5F3}">
   <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2253,99 +2240,99 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7" s="16"/>
+      <c r="C7" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="22"/>
+      <c r="C8" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="24"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="18"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B10" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="16"/>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="18"/>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="16"/>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B13" s="20"/>
+      <c r="C13" s="31" t="s">
         <v>56</v>
-      </c>
-      <c r="D9" s="16"/>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="26"/>
-    </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="16"/>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="D12" s="26"/>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="24"/>
-      <c r="C13" s="31" t="s">
-        <v>60</v>
       </c>
       <c r="D13" s="32"/>
     </row>
@@ -2353,13 +2340,13 @@
       <c r="B14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="D14" s="16"/>
+      <c r="C14" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="18"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -2370,66 +2357,66 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="12" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12"/>
       <c r="D19" s="13" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="16"/>
+      <c r="C20" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="B21" s="33"/>
+      <c r="C21" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B15:B19"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2437,18 +2424,18 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D90E38EB-7B3C-46C2-A9D2-6C84592CC87B}">
   <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2462,99 +2449,99 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>143</v>
-      </c>
-      <c r="D5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>144</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D7" s="16"/>
+      <c r="C7" s="17" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>146</v>
-      </c>
-      <c r="D8" s="16"/>
+      <c r="C8" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D8" s="18"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="D10" s="26"/>
+      <c r="C10" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
-        <v>148</v>
-      </c>
-      <c r="D11" s="16"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12" s="16"/>
+      <c r="C12" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="18"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -2565,101 +2552,101 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="18"/>
+      <c r="B14" s="26"/>
       <c r="C14" s="4" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="4" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="6" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>155</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
-        <v>156</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>151</v>
-      </c>
-      <c r="D20" s="16"/>
+      <c r="C20" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE7FC392-1A2F-41D1-A1C9-85F85E75A95B}">
   <dimension ref="B2:D25"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -2673,106 +2660,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="16"/>
+      <c r="C2" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="18"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D3" s="16"/>
+      <c r="C3" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="18"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="16"/>
+      <c r="C4" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="18"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="24"/>
-      <c r="C5" s="27" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="28"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="22"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="D6" s="26"/>
+      <c r="C6" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="D7" s="16"/>
+      <c r="C7" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="18"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" s="16"/>
+      <c r="C8" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="18"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" s="16"/>
+      <c r="C9" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="18"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" s="26"/>
+      <c r="C10" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="24"/>
-      <c r="C11" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="16"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="18"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="24"/>
-      <c r="C12" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="26"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="16"/>
+      <c r="C13" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="D13" s="18"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -2783,75 +2770,74 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="18"/>
+      <c r="B15" s="26"/>
       <c r="C15" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="18"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="18"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="12" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="18"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="19"/>
+      <c r="B19" s="27"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="D20" s="16"/>
+      <c r="C20" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D20" s="18"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="20"/>
-      <c r="C21" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D21" s="16"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="18"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2859,11 +2845,12 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Recreated code template, added sequence diagrams (almost complete) and minor fixes on other diagrams.,
</commit_message>
<xml_diff>
--- a/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
+++ b/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\SLC\TPA Desktop\DESKTOP-NB-242\Diagram\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8210BE4E-4D0A-4F33-92AA-1AF86B0A9A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7EF549-9D76-49BD-B3ED-ED07C2DC13BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="3" activeTab="7" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="2" activeTab="2" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Edit Restaurant Details" sheetId="1" r:id="rId1"/>
@@ -742,16 +742,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -765,38 +774,29 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1123,106 +1123,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1233,7 +1233,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1242,7 +1242,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="6" t="s">
         <v>25</v>
       </c>
@@ -1251,7 +1251,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="6" t="s">
         <v>28</v>
       </c>
@@ -1260,7 +1260,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="6" t="s">
         <v>29</v>
       </c>
@@ -1269,72 +1269,79 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="26"/>
+      <c r="B19" s="18"/>
       <c r="C19" s="6"/>
       <c r="D19" s="5" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="26"/>
+      <c r="B20" s="18"/>
       <c r="C20" s="6"/>
       <c r="D20" s="5" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="26"/>
+      <c r="B21" s="18"/>
       <c r="C21" s="6"/>
       <c r="D21" s="5" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B22" s="27"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="6"/>
       <c r="D22" s="5" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="18"/>
+      <c r="D23" s="16"/>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B24" s="26"/>
-      <c r="C24" s="17" t="s">
+      <c r="B24" s="18"/>
+      <c r="C24" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="D24" s="18"/>
+      <c r="D24" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B25" s="26"/>
-      <c r="C25" s="17" t="s">
+      <c r="B25" s="18"/>
+      <c r="C25" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="D25" s="18"/>
+      <c r="D25" s="16"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B26" s="26"/>
-      <c r="C26" s="17" t="s">
+      <c r="B26" s="18"/>
+      <c r="C26" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="D26" s="18"/>
+      <c r="D26" s="16"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B27" s="27"/>
-      <c r="C27" s="17" t="s">
+      <c r="B27" s="19"/>
+      <c r="C27" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="D27" s="18"/>
+      <c r="D27" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="B14:B22"/>
@@ -1349,13 +1356,6 @@
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1375,106 +1375,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -1485,7 +1485,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
@@ -1494,7 +1494,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="6" t="s">
         <v>72</v>
       </c>
@@ -1503,7 +1503,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="12" t="s">
         <v>91</v>
       </c>
@@ -1512,7 +1512,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="12" t="s">
         <v>73</v>
       </c>
@@ -1521,38 +1521,39 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="27"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="18"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="28"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="D21" s="18"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -1560,12 +1561,11 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1585,92 +1585,92 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="17" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="D5" s="18"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="2:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="24"/>
+      <c r="D6" s="28"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="28"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B10" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1681,7 +1681,7 @@
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="26"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="11" t="s">
         <v>115</v>
       </c>
@@ -1690,7 +1690,7 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="26"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="12" t="s">
         <v>116</v>
       </c>
@@ -1699,7 +1699,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="12" t="s">
         <v>118</v>
       </c>
@@ -1708,7 +1708,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="12" t="s">
         <v>119</v>
       </c>
@@ -1717,7 +1717,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="27"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="12"/>
       <c r="D17" s="11" t="s">
         <v>120</v>
@@ -1727,10 +1727,10 @@
       <c r="B18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="D18" s="18"/>
+      <c r="D18" s="16"/>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C22" s="10"/>
@@ -1742,6 +1742,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B12:B17"/>
     <mergeCell ref="C18:D18"/>
@@ -1749,12 +1755,6 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1774,106 +1774,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="28"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -1884,7 +1884,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="11" t="s">
         <v>151</v>
       </c>
@@ -1893,7 +1893,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="12" t="s">
         <v>104</v>
       </c>
@@ -1902,7 +1902,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="12" t="s">
         <v>102</v>
       </c>
@@ -1911,7 +1911,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="12" t="s">
         <v>103</v>
       </c>
@@ -1920,38 +1920,39 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="27"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="D20" s="18"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="28"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="D21" s="18"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -1959,12 +1960,11 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1984,106 +1984,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="28"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -2094,7 +2094,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
         <v>42</v>
       </c>
@@ -2103,7 +2103,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="9" t="s">
         <v>25</v>
       </c>
@@ -2112,7 +2112,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="6" t="s">
         <v>28</v>
       </c>
@@ -2121,7 +2121,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="29" t="s">
         <v>162</v>
       </c>
@@ -2130,75 +2130,86 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="26"/>
-      <c r="C19" s="34"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="30"/>
       <c r="D19" s="5" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="26"/>
-      <c r="C20" s="34"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="30"/>
       <c r="D20" s="5" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="26"/>
-      <c r="C21" s="34"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="30"/>
       <c r="D21" s="5" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B22" s="27"/>
-      <c r="C22" s="30"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="31"/>
       <c r="D22" s="5" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="18"/>
+      <c r="D23" s="16"/>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B24" s="26"/>
-      <c r="C24" s="17" t="s">
+      <c r="B24" s="18"/>
+      <c r="C24" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="D24" s="18"/>
+      <c r="D24" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B25" s="26"/>
-      <c r="C25" s="17" t="s">
+      <c r="B25" s="18"/>
+      <c r="C25" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="D25" s="18"/>
+      <c r="D25" s="16"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B26" s="26"/>
-      <c r="C26" s="17" t="s">
+      <c r="B26" s="18"/>
+      <c r="C26" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D26" s="18"/>
+      <c r="D26" s="16"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B27" s="27"/>
-      <c r="C27" s="17" t="s">
+      <c r="B27" s="19"/>
+      <c r="C27" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="D27" s="18"/>
+      <c r="D27" s="16"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C29" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:D10"/>
     <mergeCell ref="B14:B22"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C24:D24"/>
@@ -2210,17 +2221,6 @@
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2240,113 +2240,113 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="D8" s="24"/>
+      <c r="D8" s="28"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="20"/>
-      <c r="C13" s="31" t="s">
+      <c r="B13" s="23"/>
+      <c r="C13" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="32"/>
+      <c r="D13" s="34"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="18"/>
+      <c r="D14" s="16"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -2357,7 +2357,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="12" t="s">
         <v>58</v>
       </c>
@@ -2366,7 +2366,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="12" t="s">
         <v>61</v>
       </c>
@@ -2375,7 +2375,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="12" t="s">
         <v>62</v>
       </c>
@@ -2384,39 +2384,39 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="27"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="12"/>
       <c r="D19" s="13" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="18"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="33"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="32"/>
+      <c r="C21" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="D21" s="18"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B15:B19"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2424,12 +2424,12 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B15:B19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2449,99 +2449,99 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>123</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D12" s="18"/>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="14" t="s">
@@ -2552,7 +2552,7 @@
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="26"/>
+      <c r="B14" s="18"/>
       <c r="C14" s="4" t="s">
         <v>171</v>
       </c>
@@ -2561,7 +2561,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
         <v>172</v>
       </c>
@@ -2570,7 +2570,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="6" t="s">
         <v>127</v>
       </c>
@@ -2579,7 +2579,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="12" t="s">
         <v>128</v>
       </c>
@@ -2588,7 +2588,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="12" t="s">
         <v>126</v>
       </c>
@@ -2597,50 +2597,50 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="27"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D20" s="18"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="28"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="18"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="B13:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2660,106 +2660,106 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D2" s="18"/>
+      <c r="D2" s="16"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="D3" s="18"/>
+      <c r="D3" s="16"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="18"/>
+      <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="D6" s="16"/>
+      <c r="D6" s="21"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="D7" s="18"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="D8" s="18"/>
+      <c r="D8" s="16"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="18"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D10" s="16"/>
+      <c r="D10" s="21"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B11" s="20"/>
-      <c r="C11" s="17" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="18"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B12" s="20"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="23"/>
+      <c r="C12" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="16"/>
+      <c r="D12" s="21"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="17" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="14" t="s">
@@ -2770,7 +2770,7 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B15" s="26"/>
+      <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
         <v>88</v>
       </c>
@@ -2779,7 +2779,7 @@
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="26"/>
+      <c r="B16" s="18"/>
       <c r="C16" s="6" t="s">
         <v>72</v>
       </c>
@@ -2788,7 +2788,7 @@
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
-      <c r="B17" s="26"/>
+      <c r="B17" s="18"/>
       <c r="C17" s="12" t="s">
         <v>92</v>
       </c>
@@ -2797,7 +2797,7 @@
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B18" s="26"/>
+      <c r="B18" s="18"/>
       <c r="C18" s="12" t="s">
         <v>73</v>
       </c>
@@ -2806,38 +2806,39 @@
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B19" s="27"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="12"/>
       <c r="D19" s="11" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="18"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B21" s="28"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="26"/>
+      <c r="C21" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="18"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C25" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C9:D9"/>
@@ -2845,12 +2846,11 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finished Sequence, Started on Class
</commit_message>
<xml_diff>
--- a/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
+++ b/Diagram/NB_TPA_Desktop_UseCaseDescription.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\SLC\TPA Desktop\DESKTOP-NB-242\Diagram\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7EF549-9D76-49BD-B3ED-ED07C2DC13BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4160165B-F460-49ED-9492-C218F4A5933F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="2" activeTab="2" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="771" firstSheet="2" activeTab="5" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Edit Restaurant Details" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="176">
   <si>
     <t>Use Case Name:</t>
   </si>
@@ -460,9 +460,6 @@
   </si>
   <si>
     <t>4.1 Unavailable staff assigned, staff already assigned, staff on leave, etc.</t>
-  </si>
-  <si>
-    <t>V</t>
   </si>
   <si>
     <t>2. Customer Service Manager wants to send a broadcast message to notify people of an announcement.</t>
@@ -1573,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB3C5E41-754C-46AC-8647-361E83105886}">
-  <dimension ref="B2:D26"/>
+  <dimension ref="B2:D22"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.58203125" bestFit="1" customWidth="1"/>
@@ -1611,7 +1608,7 @@
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" s="23"/>
       <c r="C5" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" s="16"/>
     </row>
@@ -1713,7 +1710,7 @@
         <v>119</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.35">
@@ -1728,17 +1725,12 @@
         <v>12</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D18" s="16"/>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="C22" s="10"/>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="C26" t="s">
-        <v>139</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1793,14 +1785,14 @@
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" s="23"/>
       <c r="C5" s="24" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D5" s="25"/>
     </row>
@@ -1809,7 +1801,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D6" s="21"/>
     </row>
@@ -1827,7 +1819,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D8" s="28"/>
     </row>
@@ -1852,14 +1844,14 @@
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="23"/>
       <c r="C11" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D11" s="16"/>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B12" s="23"/>
       <c r="C12" s="20" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D12" s="21"/>
     </row>
@@ -1886,10 +1878,10 @@
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B15" s="18"/>
       <c r="C15" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D15" s="11" t="s">
         <v>151</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.35">
@@ -1931,14 +1923,14 @@
         <v>12</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D20" s="16"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="26"/>
       <c r="C21" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D21" s="16"/>
     </row>
@@ -2123,38 +2115,38 @@
     <row r="18" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B18" s="18"/>
       <c r="C18" s="29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B19" s="18"/>
       <c r="C19" s="30"/>
       <c r="D19" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B20" s="18"/>
       <c r="C20" s="30"/>
       <c r="D20" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="18"/>
       <c r="C21" s="30"/>
       <c r="D21" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B22" s="19"/>
       <c r="C22" s="31"/>
       <c r="D22" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.35">
@@ -2169,28 +2161,28 @@
     <row r="24" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B24" s="18"/>
       <c r="C24" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D24" s="16"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B25" s="18"/>
       <c r="C25" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D25" s="16"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B26" s="18"/>
       <c r="C26" s="15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D26" s="16"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B27" s="19"/>
       <c r="C27" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D27" s="16"/>
     </row>
@@ -2402,7 +2394,7 @@
     <row r="21" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B21" s="32"/>
       <c r="C21" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D21" s="16"/>
     </row>
@@ -2450,7 +2442,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D2" s="16"/>
     </row>
@@ -2459,7 +2451,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D3" s="16"/>
     </row>
@@ -2468,14 +2460,14 @@
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D4" s="16"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" s="23"/>
       <c r="C5" s="24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D5" s="25"/>
     </row>
@@ -2484,7 +2476,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D6" s="21"/>
     </row>
@@ -2502,7 +2494,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D8" s="16"/>
     </row>
@@ -2527,7 +2519,7 @@
     <row r="11" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B11" s="23"/>
       <c r="C11" s="15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D11" s="16"/>
     </row>
@@ -2554,19 +2546,19 @@
     <row r="14" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B14" s="18"/>
       <c r="C14" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B15" s="18"/>
       <c r="C15" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2575,7 +2567,7 @@
         <v>127</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="31" x14ac:dyDescent="0.35">
@@ -2608,7 +2600,7 @@
         <v>12</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D20" s="16"/>
     </row>

</xml_diff>